<commit_message>
Simulador de pinpad, pago de adeudos en conjunto y estado de 6 MSI
- v1.6.37 usa el simulador de pinpad de Memphis: la suite lo detecta y toca
  Approved/Declined (FlujoKiosko.completar_cobro), así corren desatendidos el
  happy path, rechazo, comprobante, reimpresión, datos enmascarados,
  referencia repetida, fecha/hora, notificación y cambio de red.
- Todo pago aprobado marca la referencia como 'pagada' automáticamente.
- Nuevo comprobante P5 (folio, total, autorización, tarjeta, fecha).
- Casos de tarjeta física (chip, banda, NIP, contactless, timeout, cancelar)
  y 6 MSI quedan Pendientes: falta la animación de tarjeta / NIP.
- Regla de negocio: los adeudos se pagan siempre en conjunto (CP-AD-ROM-001
  a 003 y textos de la matriz ajustados).
- Catálogo: referencias pagadas en las pruebas del 15/10/2026.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/RompeFilas.xlsx
+++ b/data/RompeFilas.xlsx
@@ -4422,32 +4422,32 @@
       </c>
       <c r="G17" s="45" t="inlineStr">
         <is>
-          <t>Selección de un adeudo individual</t>
+          <t>Pago en conjunto de todos los adeudos (sin selección individual)</t>
         </is>
       </c>
       <c r="H17" s="45" t="inlineStr">
         <is>
-          <t>Validar: Selección de un adeudo individual</t>
+          <t>Validar: Pago en conjunto de todos los adeudos (sin selección individual)</t>
         </is>
       </c>
       <c r="I17" s="46" t="inlineStr">
         <is>
-          <t>P2 visible con 4 adeudos (Predial Urbano, Recargos x2, Limpia).
+          <t>P2 visible con los adeudos de la referencia (ej. Predial Urbano, Recargos x2, Limpia).
 Datos de prueba:
-1 adeudo — $100.00</t>
+Referencia 'disponible' del catálogo — total de todos sus adeudos</t>
         </is>
       </c>
       <c r="J17" s="45" t="inlineStr">
         <is>
           <t>1. Desplazar (scroll) la lista si es necesario.
-2. Tocar la casilla 'PREDIAL URBANO $100.00'.
-3. Verificar total actualizado.
-4. Presionar 'Pagar ahora'.</t>
+2. Verificar que no haya casillas para elegir adeudos individuales.
+3. Presionar 'Pagar ahora'.
+4. Verificar el total en P3.</t>
         </is>
       </c>
       <c r="K17" s="45" t="inlineStr">
         <is>
-          <t>La lista es desplazable en la pantalla de la T6, los conceptos y montos no se truncan, el total se actualiza a $100.00 y avanza a P3.</t>
+          <t>La lista es desplazable, los conceptos y montos no se truncan, no es posible seleccionar adeudos individuales y P3 cobra la suma de TODOS los adeudos.</t>
         </is>
       </c>
       <c r="L17" s="47" t="inlineStr">
@@ -4491,7 +4491,11 @@
         </is>
       </c>
       <c r="U17" s="44" t="n"/>
-      <c r="V17" s="52" t="n"/>
+      <c r="V17" s="52" t="inlineStr">
+        <is>
+          <t>Ajuste 15/10/2026: los adeudos no se pagan de forma individual; siempre se pagan todos en conjunto.</t>
+        </is>
+      </c>
       <c r="W17" s="40" t="n"/>
       <c r="X17" s="40" t="n"/>
       <c r="Y17" s="40" t="n"/>
@@ -4536,12 +4540,12 @@
       </c>
       <c r="G18" s="45" t="inlineStr">
         <is>
-          <t>Selección de todos los adeudos con 'Seleccionar todo'</t>
+          <t>Todos los adeudos se incluyen automáticamente en el pago</t>
         </is>
       </c>
       <c r="H18" s="45" t="inlineStr">
         <is>
-          <t>Validar: Selección de todos los adeudos con 'Seleccionar todo'</t>
+          <t>Validar: Todos los adeudos se incluyen automáticamente en el pago</t>
         </is>
       </c>
       <c r="I18" s="46" t="inlineStr">
@@ -4553,14 +4557,14 @@
       </c>
       <c r="J18" s="45" t="inlineStr">
         <is>
-          <t>1. Tocar 'Seleccionar todo'.
-2. Verificar que los 4 adeudos queden marcados (incluyendo los que quedan fuera de la vista).
-3. Presionar 'Pagar ahora'.</t>
+          <t>1. Revisar la lista de adeudos en P2 (incluyendo los que quedan fuera de la vista).
+2. Presionar 'Pagar ahora'.
+3. Verificar el total en P3.</t>
         </is>
       </c>
       <c r="K18" s="45" t="inlineStr">
         <is>
-          <t>Los 4 adeudos quedan marcados, el total = $500.00 MXN es correcto y visible, y avanza a P3.</t>
+          <t>Todos los adeudos quedan incluidos sin acción del usuario (no hay 'Seleccionar todo'); el total en P3 es la suma de todos y es correcto y visible.</t>
         </is>
       </c>
       <c r="L18" s="47" t="inlineStr">
@@ -4604,7 +4608,11 @@
         </is>
       </c>
       <c r="U18" s="44" t="n"/>
-      <c r="V18" s="52" t="n"/>
+      <c r="V18" s="52" t="inlineStr">
+        <is>
+          <t>Ajuste 15/10/2026: los adeudos no se pagan de forma individual; siempre se pagan todos en conjunto.</t>
+        </is>
+      </c>
       <c r="W18" s="40" t="n"/>
       <c r="X18" s="40" t="n"/>
       <c r="Y18" s="40" t="n"/>
@@ -4649,30 +4657,30 @@
       </c>
       <c r="G19" s="45" t="inlineStr">
         <is>
-          <t>Intentar avanzar sin seleccionar ningún adeudo</t>
+          <t>No es posible quitar adeudos ni cobrar $0.00</t>
         </is>
       </c>
       <c r="H19" s="45" t="inlineStr">
         <is>
-          <t>Validar: Intentar avanzar sin seleccionar ningún adeudo</t>
+          <t>Validar: No es posible quitar adeudos ni cobrar $0.00</t>
         </is>
       </c>
       <c r="I19" s="46" t="inlineStr">
         <is>
-          <t>P2 visible. Ninguna casilla marcada.
+          <t>P2 visible con adeudos cargados.
 Datos de prueba:
-0 adeudos — $0.00</t>
+Referencia 'disponible' del catálogo</t>
         </is>
       </c>
       <c r="J19" s="45" t="inlineStr">
         <is>
-          <t>1. No tocar ningún adeudo.
+          <t>1. Intentar desmarcar o quitar adeudos de la lista.
 2. Presionar 'Pagar ahora'.</t>
         </is>
       </c>
       <c r="K19" s="45" t="inlineStr">
         <is>
-          <t>El botón 'Pagar ahora' está deshabilitado o se muestra aviso; no se avanza a P3.</t>
+          <t>No hay forma de quitar adeudos; 'Pagar ahora' siempre cobra el total de la referencia (nunca $0.00).</t>
         </is>
       </c>
       <c r="L19" s="47" t="inlineStr">
@@ -4716,7 +4724,11 @@
         </is>
       </c>
       <c r="U19" s="44" t="n"/>
-      <c r="V19" s="52" t="n"/>
+      <c r="V19" s="52" t="inlineStr">
+        <is>
+          <t>Ajuste 15/10/2026: los adeudos no se pagan de forma individual; siempre se pagan todos en conjunto.</t>
+        </is>
+      </c>
       <c r="W19" s="40" t="n"/>
       <c r="X19" s="40" t="n"/>
       <c r="Y19" s="40" t="n"/>
@@ -4884,7 +4896,7 @@
       </c>
       <c r="I21" s="46" t="inlineStr">
         <is>
-          <t>P3 visible. 1 adeudo seleccionado ($100.00).
+          <t>P3 visible con el total de la referencia (todos los adeudos, en conjunto).
 Datos de prueba:
 Método: Tarjeta</t>
         </is>
@@ -4896,7 +4908,7 @@
       </c>
       <c r="K21" s="45" t="inlineStr">
         <is>
-          <t>La app invoca el módulo de pago integrado de la T6 (sin terminal externa), muestra el monto $100.00 y la instrucción para insertar, deslizar o acercar la tarjeta.</t>
+          <t>La app invoca el módulo de pago integrado de la T6 (sin terminal externa), muestra el monto total y la instrucción para insertar, deslizar o acercar la tarjeta.</t>
         </is>
       </c>
       <c r="L21" s="47" t="inlineStr">
@@ -4995,7 +5007,7 @@
       </c>
       <c r="I22" s="46" t="inlineStr">
         <is>
-          <t>Pantalla de cobro activa en la T6 con monto $100.00.
+          <t>Pantalla de cobro activa en la T6 con el total de la referencia (todos los adeudos, en conjunto).
 Datos de prueba:
 Tarjeta débito Visa/Mastercard con fondos</t>
         </is>
@@ -5334,7 +5346,7 @@
         <is>
           <t>Pago aprobado. Rollo de papel cargado en la T6.
 Datos de prueba:
-Pago $100 completado</t>
+Pago completado por el total de la referencia (todos los adeudos, en conjunto)</t>
         </is>
       </c>
       <c r="J25" s="45" t="inlineStr">
@@ -5447,7 +5459,7 @@
         <is>
           <t>Pago con tarjeta aprobado. Papel disponible.
 Datos de prueba:
-Pago $100 con tarjeta</t>
+Pago con tarjeta por el total de la referencia (todos los adeudos, en conjunto)</t>
         </is>
       </c>
       <c r="J26" s="45" t="inlineStr">
@@ -7244,7 +7256,7 @@
       </c>
       <c r="I42" s="46" t="inlineStr">
         <is>
-          <t>Pantalla de cobro activa con monto $100.00.
+          <t>Pantalla de cobro activa con el total de la referencia (todos los adeudos, en conjunto).
 Datos de prueba:
 Tarjeta crédito Visa/Mastercard</t>
         </is>
@@ -7357,9 +7369,9 @@
       </c>
       <c r="I43" s="46" t="inlineStr">
         <is>
-          <t>Pantalla de cobro activa. Monto menor al límite contactless del adquirente.
+          <t>Pantalla de cobro activa. Total de la referencia (todos los adeudos) menor al límite contactless del adquirente.
 Datos de prueba:
-Tarjeta/Wallet NFC — $100.00</t>
+Tarjeta/Wallet NFC</t>
         </is>
       </c>
       <c r="J43" s="45" t="inlineStr">
@@ -9710,7 +9722,7 @@
       </c>
       <c r="J64" s="45" t="inlineStr">
         <is>
-          <t>1. Seleccionar el mismo adeudo en ambos dispositivos.
+          <t>1. Consultar la misma referencia en ambos dispositivos (se pagan todos sus adeudos en conjunto).
 2. Pagar primero en el Tótem.
 3. Intentar pagar en la T6.</t>
         </is>
@@ -9816,7 +9828,7 @@
       </c>
       <c r="I65" s="46" t="inlineStr">
         <is>
-          <t>P2/P3 con adeudo seleccionado.
+          <t>P2/P3 con los adeudos de la referencia (todos, en conjunto).
 Datos de prueba:
 Doble toque</t>
         </is>
@@ -11219,7 +11231,7 @@
       <c r="U77" s="44" t="n"/>
       <c r="V77" s="52" t="inlineStr">
         <is>
-          <t>6 MSI: aplica a transacciones a partir de $1,000.00. Validación manual.</t>
+          <t>6 MSI: aplica a transacciones a partir de $1,000.00. Validación manual. Aún NO integrado en v1.6.37: falta la animación para insertar la tarjeta y capturar el NIP.</t>
         </is>
       </c>
       <c r="W77" s="40" t="n"/>
@@ -11338,7 +11350,7 @@
       <c r="U78" s="44" t="n"/>
       <c r="V78" s="52" t="inlineStr">
         <is>
-          <t>6 MSI: aplica a transacciones a partir de $1,000.00. Validación manual.</t>
+          <t>6 MSI: aplica a transacciones a partir de $1,000.00. Validación manual. Aún NO integrado en v1.6.37: falta la animación para insertar la tarjeta y capturar el NIP.</t>
         </is>
       </c>
       <c r="W78" s="40" t="n"/>
@@ -11457,7 +11469,7 @@
       <c r="U79" s="44" t="n"/>
       <c r="V79" s="52" t="inlineStr">
         <is>
-          <t>6 MSI: aplica a transacciones a partir de $1,000.00. Validación manual.</t>
+          <t>6 MSI: aplica a transacciones a partir de $1,000.00. Validación manual. Aún NO integrado en v1.6.37: falta la animación para insertar la tarjeta y capturar el NIP.</t>
         </is>
       </c>
       <c r="W79" s="40" t="n"/>
@@ -11576,7 +11588,7 @@
       <c r="U80" s="44" t="n"/>
       <c r="V80" s="52" t="inlineStr">
         <is>
-          <t>6 MSI: aplica a transacciones a partir de $1,000.00. Validación manual.</t>
+          <t>6 MSI: aplica a transacciones a partir de $1,000.00. Validación manual. Aún NO integrado en v1.6.37: falta la animación para insertar la tarjeta y capturar el NIP.</t>
         </is>
       </c>
       <c r="W80" s="40" t="n"/>
@@ -11693,7 +11705,7 @@
       <c r="U81" s="44" t="n"/>
       <c r="V81" s="52" t="inlineStr">
         <is>
-          <t>6 MSI: aplica a transacciones a partir de $1,000.00. Validación manual.</t>
+          <t>6 MSI: aplica a transacciones a partir de $1,000.00. Validación manual. Aún NO integrado en v1.6.37: falta la animación para insertar la tarjeta y capturar el NIP.</t>
         </is>
       </c>
       <c r="W81" s="40" t="n"/>
@@ -11812,7 +11824,7 @@
       <c r="U82" s="44" t="n"/>
       <c r="V82" s="52" t="inlineStr">
         <is>
-          <t>6 MSI: aplica a transacciones a partir de $1,000.00. Validación manual.</t>
+          <t>6 MSI: aplica a transacciones a partir de $1,000.00. Validación manual. Aún NO integrado en v1.6.37: falta la animación para insertar la tarjeta y capturar el NIP.</t>
         </is>
       </c>
       <c r="W82" s="40" t="n"/>

</xml_diff>

<commit_message>
Dashboard de la matriz: incluye pruebas automatizadas
- Bloque 'Pruebas Automatizadas' (filas 35-45) y totales del sprint = manuales + automatizados
  (antes sumaban celdas H vacías bajo la gráfica y solo contaban los manuales).
- 'Sin Ejecutar' descuenta los bloqueados; Pass Rate con IFERROR (sin #DIV/0!).
- Se quita la referencia circular de D9 y se ajusta la altura del título.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/RompeFilas.xlsx
+++ b/data/RompeFilas.xlsx
@@ -1396,7 +1396,7 @@
       <c r="C1" s="54" t="n"/>
       <c r="I1" s="56" t="n"/>
     </row>
-    <row r="2" ht="15.75" customHeight="1" s="96">
+    <row r="2" ht="48" customHeight="1" s="96">
       <c r="A2" s="54" t="n"/>
       <c r="B2" s="57" t="n"/>
       <c r="C2" s="97" t="inlineStr">
@@ -1449,7 +1449,7 @@
       <c r="B9" s="55" t="n"/>
       <c r="C9" s="54" t="n"/>
       <c r="D9" s="98">
-        <f>IF(AND($E$14=0, $E$10&gt;0, $D$9&lt;&gt;""), $D$9, "Sprint: (" &amp; TEXT(TODAY() - WEEKDAY(TODAY(), 2) + 1, "dd/mm/yyyy") &amp; " - " &amp; TEXT(TODAY() - WEEKDAY(TODAY(), 2) + 5, "dd/mm/yyyy") &amp; ")")</f>
+        <f>"Sprint: (" &amp; TEXT(TODAY() - WEEKDAY(TODAY(), 2) + 1, "dd/mm/yyyy") &amp; " - " &amp; TEXT(TODAY() - WEEKDAY(TODAY(), 2) + 5, "dd/mm/yyyy") &amp; ")"</f>
         <v/>
       </c>
       <c r="E9" s="99" t="n"/>
@@ -1465,7 +1465,7 @@
         </is>
       </c>
       <c r="E10" s="63">
-        <f>$D$22+$H$22</f>
+        <f>$D$22+$D$35</f>
         <v/>
       </c>
       <c r="I10" s="56" t="n"/>
@@ -1480,7 +1480,7 @@
         </is>
       </c>
       <c r="E11" s="63">
-        <f>$D$29+$H$29</f>
+        <f>$D$29+$D$42</f>
         <v/>
       </c>
       <c r="I11" s="56" t="n"/>
@@ -1495,7 +1495,7 @@
         </is>
       </c>
       <c r="E12" s="64">
-        <f>$D$30+$H$30</f>
+        <f>$D$30+$D$43</f>
         <v/>
       </c>
       <c r="I12" s="56" t="n"/>
@@ -1510,7 +1510,7 @@
         </is>
       </c>
       <c r="E13" s="65">
-        <f>$D$31+$H$31</f>
+        <f>$D$31+$D$44</f>
         <v/>
       </c>
       <c r="I13" s="56" t="n"/>
@@ -1525,7 +1525,7 @@
         </is>
       </c>
       <c r="E14" s="63">
-        <f>E10-E11-E12</f>
+        <f>E10-E11-E12-E13</f>
         <v/>
       </c>
       <c r="I14" s="56" t="n"/>
@@ -1628,7 +1628,7 @@
         </is>
       </c>
       <c r="D24" s="79">
-        <f>D29/D23</f>
+        <f>IFERROR(D29/D23,0)</f>
         <v/>
       </c>
       <c r="F24" s="69" t="n"/>
@@ -1771,28 +1771,50 @@
     </row>
     <row r="35" ht="15.75" customHeight="1" s="96">
       <c r="A35" s="54" t="n"/>
-      <c r="B35" s="55" t="n"/>
-      <c r="C35" s="54" t="n"/>
+      <c r="B35" s="71" t="n"/>
+      <c r="C35" s="72" t="inlineStr">
+        <is>
+          <t>Total de Casos Automatizados</t>
+        </is>
+      </c>
+      <c r="D35" s="73">
+        <f>SUM('Matriz Casos de Prueba Puebla'!E84)</f>
+        <v/>
+      </c>
       <c r="I35" s="56" t="n"/>
     </row>
     <row r="36" ht="15.75" customHeight="1" s="96">
       <c r="A36" s="54" t="n"/>
-      <c r="B36" s="55" t="n"/>
-      <c r="C36" s="54" t="n"/>
+      <c r="B36" s="71" t="n"/>
+      <c r="C36" s="76" t="inlineStr">
+        <is>
+          <t>Casos Automatizados Ejecutados</t>
+        </is>
+      </c>
+      <c r="D36" s="77">
+        <f>SUM('Matriz Casos de Prueba Puebla'!E88)</f>
+        <v/>
+      </c>
       <c r="I36" s="56" t="n"/>
     </row>
     <row r="37" ht="15.75" customHeight="1" s="96">
       <c r="A37" s="54" t="n"/>
-      <c r="B37" s="55" t="n"/>
-      <c r="C37" s="54" t="n"/>
+      <c r="B37" s="71" t="n"/>
+      <c r="C37" s="78" t="inlineStr">
+        <is>
+          <t>Porcentaje de Paso (Pass Rate)</t>
+        </is>
+      </c>
+      <c r="D37" s="79">
+        <f>IFERROR(D42/D36,0)</f>
+        <v/>
+      </c>
       <c r="I37" s="56" t="n"/>
     </row>
     <row r="38" ht="15.75" customHeight="1" s="96">
       <c r="A38" s="54" t="n"/>
-      <c r="B38" s="90" t="n"/>
-      <c r="C38" s="91" t="n"/>
-      <c r="D38" s="91" t="n"/>
-      <c r="E38" s="91" t="n"/>
+      <c r="B38" s="68" t="n"/>
+      <c r="C38" s="54" t="n"/>
       <c r="F38" s="91" t="n"/>
       <c r="G38" s="91" t="n"/>
       <c r="H38" s="91" t="n"/>
@@ -1800,24 +1822,84 @@
     </row>
     <row r="39" ht="15.75" customHeight="1" s="96">
       <c r="A39" s="54" t="n"/>
+      <c r="B39" s="71" t="n"/>
+      <c r="C39" s="54" t="n"/>
     </row>
     <row r="40" ht="15.75" customHeight="1" s="96">
       <c r="A40" s="54" t="n"/>
+      <c r="B40" s="71" t="n"/>
+      <c r="C40" s="81" t="inlineStr">
+        <is>
+          <t>Resultado de Ejecución de Pruebas Automatizadas</t>
+        </is>
+      </c>
+      <c r="D40" s="82" t="n"/>
     </row>
     <row r="41" ht="15.75" customHeight="1" s="96">
       <c r="A41" s="54" t="n"/>
+      <c r="B41" s="71" t="n"/>
+      <c r="C41" s="84" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="D41" s="85" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="15.75" customHeight="1" s="96">
       <c r="A42" s="54" t="n"/>
+      <c r="B42" s="71" t="n"/>
+      <c r="C42" s="76" t="inlineStr">
+        <is>
+          <t>Pasó</t>
+        </is>
+      </c>
+      <c r="D42" s="87">
+        <f>'Matriz Casos de Prueba Puebla'!E85</f>
+        <v/>
+      </c>
     </row>
     <row r="43" ht="15.75" customHeight="1" s="96">
       <c r="A43" s="54" t="n"/>
+      <c r="B43" s="71" t="n"/>
+      <c r="C43" s="76" t="inlineStr">
+        <is>
+          <t>Falló</t>
+        </is>
+      </c>
+      <c r="D43" s="87">
+        <f>'Matriz Casos de Prueba Puebla'!E86</f>
+        <v/>
+      </c>
     </row>
     <row r="44" ht="15.75" customHeight="1" s="96">
       <c r="A44" s="54" t="n"/>
+      <c r="B44" s="71" t="n"/>
+      <c r="C44" s="76" t="inlineStr">
+        <is>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="D44" s="87">
+        <f>'Matriz Casos de Prueba Puebla'!E87</f>
+        <v/>
+      </c>
     </row>
     <row r="45" ht="15.75" customHeight="1" s="96">
       <c r="A45" s="54" t="n"/>
+      <c r="B45" s="71" t="n"/>
+      <c r="C45" s="78" t="inlineStr">
+        <is>
+          <t>Sin Ejecutar</t>
+        </is>
+      </c>
+      <c r="D45" s="89">
+        <f>$D$35-$D$36</f>
+        <v/>
+      </c>
     </row>
     <row r="46" ht="15.75" customHeight="1" s="96">
       <c r="A46" s="54" t="n"/>

</xml_diff>

<commit_message>
Pinpad real de Memphis: flujo guiado de tarjeta, mensualidades y NIP
- Pantallas del pinpad (inserción, lectura, mensualidades, NIP, aprobada/declinada/tiempo agotado/PIN cancelado)
  y detalle del error en Rompefilas.
- 3 min para la tarjeta y 3 min para el NIP; con montos >= $1,000 la suite elige el plan (contado o 6 MSI).
- CP-TJ-ROM-003 y CP-TJ-ROM-012 corren sin tester; 6 MSI integrado (CP-MSI-ROM-001 a 006).
- Montos negativos (condonaciones) se restan del total.
- CP-IC-ROM-002: solo falla si una actividad del módulo de pago se repite (antes daba falso positivo).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/RompeFilas.xlsx
+++ b/data/RompeFilas.xlsx
@@ -11313,7 +11313,7 @@
       <c r="U77" s="44" t="n"/>
       <c r="V77" s="52" t="inlineStr">
         <is>
-          <t>6 MSI: aplica a transacciones a partir de $1,000.00. Validación manual. Aún NO integrado en v1.6.37: falta la animación para insertar la tarjeta y capturar el NIP.</t>
+          <t>6 MSI: aplica a transacciones a partir de $1,000.00. Integrado el 27/10/2026: tras leer la tarjeta el pinpad muestra '¿Cuántas mensualidades?' (Sin mensualidades / 6 meses sin intereses) y el NIP muestra 'Mensualidades 6'. Ticket impreso: validación manual.</t>
         </is>
       </c>
       <c r="W77" s="40" t="n"/>
@@ -11432,7 +11432,7 @@
       <c r="U78" s="44" t="n"/>
       <c r="V78" s="52" t="inlineStr">
         <is>
-          <t>6 MSI: aplica a transacciones a partir de $1,000.00. Validación manual. Aún NO integrado en v1.6.37: falta la animación para insertar la tarjeta y capturar el NIP.</t>
+          <t>6 MSI: aplica a transacciones a partir de $1,000.00. Integrado el 27/10/2026: tras leer la tarjeta el pinpad muestra '¿Cuántas mensualidades?' (Sin mensualidades / 6 meses sin intereses) y el NIP muestra 'Mensualidades 6'. Ticket impreso: validación manual.</t>
         </is>
       </c>
       <c r="W78" s="40" t="n"/>
@@ -11551,7 +11551,7 @@
       <c r="U79" s="44" t="n"/>
       <c r="V79" s="52" t="inlineStr">
         <is>
-          <t>6 MSI: aplica a transacciones a partir de $1,000.00. Validación manual. Aún NO integrado en v1.6.37: falta la animación para insertar la tarjeta y capturar el NIP.</t>
+          <t>6 MSI: aplica a transacciones a partir de $1,000.00. Integrado el 27/10/2026: tras leer la tarjeta el pinpad muestra '¿Cuántas mensualidades?' (Sin mensualidades / 6 meses sin intereses) y el NIP muestra 'Mensualidades 6'. Ticket impreso: validación manual.</t>
         </is>
       </c>
       <c r="W79" s="40" t="n"/>
@@ -11670,7 +11670,7 @@
       <c r="U80" s="44" t="n"/>
       <c r="V80" s="52" t="inlineStr">
         <is>
-          <t>6 MSI: aplica a transacciones a partir de $1,000.00. Validación manual. Aún NO integrado en v1.6.37: falta la animación para insertar la tarjeta y capturar el NIP.</t>
+          <t>6 MSI: aplica a transacciones a partir de $1,000.00. Integrado el 27/10/2026: tras leer la tarjeta el pinpad muestra '¿Cuántas mensualidades?' (Sin mensualidades / 6 meses sin intereses) y el NIP muestra 'Mensualidades 6'. Ticket impreso: validación manual.</t>
         </is>
       </c>
       <c r="W80" s="40" t="n"/>
@@ -11787,7 +11787,7 @@
       <c r="U81" s="44" t="n"/>
       <c r="V81" s="52" t="inlineStr">
         <is>
-          <t>6 MSI: aplica a transacciones a partir de $1,000.00. Validación manual. Aún NO integrado en v1.6.37: falta la animación para insertar la tarjeta y capturar el NIP.</t>
+          <t>6 MSI: aplica a transacciones a partir de $1,000.00. Integrado el 27/10/2026: tras leer la tarjeta el pinpad muestra '¿Cuántas mensualidades?' (Sin mensualidades / 6 meses sin intereses) y el NIP muestra 'Mensualidades 6'. Ticket impreso: validación manual.</t>
         </is>
       </c>
       <c r="W81" s="40" t="n"/>
@@ -11906,7 +11906,7 @@
       <c r="U82" s="44" t="n"/>
       <c r="V82" s="52" t="inlineStr">
         <is>
-          <t>6 MSI: aplica a transacciones a partir de $1,000.00. Validación manual. Aún NO integrado en v1.6.37: falta la animación para insertar la tarjeta y capturar el NIP.</t>
+          <t>6 MSI: aplica a transacciones a partir de $1,000.00. Integrado el 27/10/2026: tras leer la tarjeta el pinpad muestra '¿Cuántas mensualidades?' (Sin mensualidades / 6 meses sin intereses) y el NIP muestra 'Mensualidades 6'. Ticket impreso: validación manual.</t>
         </is>
       </c>
       <c r="W82" s="40" t="n"/>

</xml_diff>